<commit_message>
fix: update sample data and improve datatype mismatch detection
- generate_sample_data.py: use consistent YYYY-MM-DD dates, remove +1 phone format, string zip codes
- transformer.py: smarter dtype detection - distinguish between Excel storage format (int64 zip codes) and rogue numeric values in text columns
- Regenerated sample_data/legacy_crm_export.xlsx
</commit_message>
<xml_diff>
--- a/sample_data/legacy_crm_export.xlsx
+++ b/sample_data/legacy_crm_export.xlsx
@@ -473,74 +473,74 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Linda Jackson</t>
+          <t>Elizabeth Lopez</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>371.383.5406</t>
+          <t>782-552-4041</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>linda.jackson@gmail.com</t>
+          <t>elizabeth.lopez@company.org</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>22-5-2005</t>
+          <t>1968-07-03</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3499 Cedar St</t>
+          <t>9220 Main St</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>82120</t>
+          <t>32921</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Linda Smith</t>
+          <t>William Anderson</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>+17595737284</t>
+          <t>(807) 740-2593</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>linda.smith@mail.co</t>
+          <t>william.anderson@mail.co</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>26.07.1980</t>
+          <t>1974-12-11</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5750 Pine St</t>
+          <t>7877 Pine St</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -550,34 +550,34 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>60572</t>
+          <t>48402</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Elizabeth Miller</t>
+          <t>Linda Jackson</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>229.776.6407</t>
+          <t>250.627.0180</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>elizabeth.miller@gmail.com</t>
+          <t>linda.jackson@mail.co</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>13.02.1969</t>
+          <t>1981-01-22</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7718 Pine St</t>
+          <t>7450 Cedar St</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -587,39 +587,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>84224</t>
+          <t>77158</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Susan Garcia</t>
+          <t>Mary Anderson</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(840) 488-2793</t>
+          <t>(823) 605-2377</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>susan.garcia@company.org</t>
+          <t>mary.anderson@yahoo.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1994-11-23</t>
+          <t>1975-07-20</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6572 Main St</t>
+          <t>9127 Cedar St</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -629,39 +629,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>33287</t>
+          <t>94644</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>David Garcia</t>
+          <t>James Miller</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>(664) 712-8722</t>
+          <t>313 585 1107</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>david.garcia@yahoo.com</t>
+          <t>james.miller@company.org</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>02.01.1980</t>
+          <t>1976-12-24</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2252 Elm St</t>
+          <t>3273 Oak St</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -671,165 +671,165 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>78880</t>
+          <t>20883</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>James Martinez</t>
+          <t>Patricia Thomas</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>347.978.4549</t>
+          <t>491-949-9559</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>james.martinez@outlook.com</t>
+          <t>patricia.thomas@company.org</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2/25/1962</t>
+          <t>1978-05-13</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>626 Main St</t>
+          <t>1510 Pine St</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>80719</t>
+          <t>77526</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sarah Smith</t>
+          <t>Elizabeth Jackson</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>362.120.6119</t>
+          <t>228.736.2969</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sarah.smith@mail.co</t>
+          <t>elizabeth.jackson@company.org</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06/14/1976</t>
+          <t>1964-01-14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8616 Oak St</t>
+          <t>8488 Cedar St</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>69803</t>
+          <t>85475</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Patricia Brown</t>
+          <t>James Martin</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>+17072344637</t>
+          <t>378.187.3007</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>patricia.brown@gmail.com</t>
+          <t>james.martin@mail.co</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15.10.1969</t>
+          <t>1961-03-15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>6728 Cedar St</t>
+          <t>2153 Main St</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>31909</t>
+          <t>75323</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jessica Miller</t>
+          <t>James Anderson</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>683.404.5526</t>
+          <t>736 638 8044</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>jessica.miller@company.org</t>
+          <t>james.anderson@mail.co</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>13-3-1994</t>
+          <t>1961-07-23</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2770 Pine St</t>
+          <t>5571 Oak St</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -839,86 +839,86 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>28479</t>
+          <t>17600</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Richard Rodriguez</t>
+          <t>Sarah Williams</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>+17368246187</t>
+          <t>698-817-9400</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>richard.rodriguez@mail.co</t>
+          <t>sarah.williams@mail.co</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1989-08-14</t>
+          <t>1999-11-02</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4955 Elm St</t>
+          <t>6886 Oak St</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>95872</t>
+          <t>61897</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jennifer Martinez</t>
+          <t>William Martin</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>421.975.2987</t>
+          <t>767-172-7319</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>jennifer.martinez@outlook.com</t>
+          <t>william.martin@yahoo.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>21.04.1992</t>
+          <t>1960-10-19</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>719 Pine St</t>
+          <t>3962 Main St</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -928,328 +928,328 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>48069</t>
+          <t>51386</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Richard Miller</t>
+          <t>Linda Williams</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>+15478259588</t>
+          <t>483 543 0317</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>richard.miller@company.org</t>
+          <t>linda.williams@outlook.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1979-01-12</t>
+          <t>1970-07-17</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8730 Pine St</t>
+          <t>3636 Elm St</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>57249</t>
+          <t>76769</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>William Jackson</t>
+          <t>Jennifer Garcia</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(889) 401-5094</t>
+          <t>728 951 7107</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>william.jackson@gmail.com</t>
+          <t>jennifer.garcia@mail.co</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14-4-2004</t>
+          <t>1967-11-20</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4365 Oak St</t>
+          <t>3263 Cedar St</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>26090</t>
+          <t>79327</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>James Anderson</t>
+          <t>Robert Wilson</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>(228) 468-1696</t>
+          <t>532 400 3498</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>james.anderson@outlook.com</t>
+          <t>robert.wilson@company.org</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>11-2-2000</t>
+          <t>1967-08-10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3743 Elm St</t>
+          <t>6554 Cedar St</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>90264</t>
+          <t>50930</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Linda Miller</t>
+          <t>Patricia Miller</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>307 171 9920</t>
+          <t>978-578-1997</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>linda.miller@company.org</t>
+          <t>patricia.miller@outlook.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3-10-2003</t>
+          <t>1986-07-10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3245 Cedar St</t>
+          <t>2365 Main St</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>76886</t>
+          <t>44407</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mary Anderson</t>
+          <t>Elizabeth Wilson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>536 340 8944</t>
+          <t>806-864-5855</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>mary.anderson@company.org</t>
+          <t>elizabeth.wilson@mail.co</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2/3/1990</t>
+          <t>1974-08-02</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1919 Oak St</t>
+          <t>3116 Oak St</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>43282</t>
+          <t>59740</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Richard Martin</t>
+          <t>Richard Miller</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>(905) 978-2345</t>
+          <t>824-204-4450</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>richard.martin@mail.co</t>
+          <t>richard.miller@outlook.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07/15/1978</t>
+          <t>1966-07-17</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4335 Oak St</t>
+          <t>6123 Elm St</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>26827</t>
+          <t>63711</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Joseph Gonzalez</t>
+          <t>Elizabeth Rodriguez</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>598-541-6868</t>
+          <t>985 980 9432</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>joseph.gonzalez@mail.co</t>
+          <t>elizabeth.rodriguez@company.org</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1/12/1984</t>
+          <t>1974-05-10</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2549 Elm St</t>
+          <t>9709 Main St</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>48551</t>
+          <t>13456</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Robert Thomas</t>
+          <t>Jennifer Lopez</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>(999) 641-8621</t>
+          <t>436 857 2426</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>robert.thomas@yahoo.com</t>
+          <t>jennifer.lopez@yahoo.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>12.07.2002</t>
+          <t>1975-07-16</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>6254 Pine St</t>
+          <t>7059 Elm St</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1259,39 +1259,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>63343</t>
+          <t>89531</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Karen Anderson</t>
+          <t>Elizabeth Garcia</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(624) 373-2899</t>
+          <t>682 466 9789</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>karen.anderson@company.org</t>
+          <t>elizabeth.garcia@yahoo.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>11/25/1970</t>
+          <t>2001-04-10</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7754 Cedar St</t>
+          <t>752 Cedar St</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1301,165 +1301,165 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>25803</t>
+          <t>79204</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Linda Anderson</t>
+          <t>Patricia Johnson</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>+12955342790</t>
+          <t>826-427-9739</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>linda.anderson@company.org</t>
+          <t>patricia.johnson@yahoo.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>04/09/1970</t>
+          <t>1966-04-22</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>6097 Main St</t>
+          <t>4544 Cedar St</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>39939</t>
+          <t>19024</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jennifer Thomas</t>
+          <t>Thomas Smith</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>+18274190698</t>
+          <t>940-416-5381</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>jennifer.thomas@gmail.com</t>
+          <t>thomas.smith@outlook.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10/14/2004</t>
+          <t>1986-08-02</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>9075 Elm St</t>
+          <t>9143 Main St</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>74700</t>
+          <t>13007</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Robert Anderson</t>
+          <t>Richard Martin</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>685-471-6510</t>
+          <t>625.425.3835</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>robert.anderson@mail.co</t>
+          <t>richard.martin@outlook.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>14-11-1996</t>
+          <t>1976-11-08</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2334 Cedar St</t>
+          <t>8067 Pine St</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>49437</t>
+          <t>91216</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Karen Lopez</t>
+          <t>Susan Brown</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>(935) 573-0935</t>
+          <t>(418) 154-1048</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>karen.lopez@gmail.com</t>
+          <t>susan.brown@yahoo.com</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4/18/1993</t>
+          <t>1964-03-18</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>8937 Cedar St</t>
+          <t>4747 Cedar St</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1469,207 +1469,207 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>49233</t>
+          <t>40815</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>David Moore</t>
+          <t>Susan Miller</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>782 473 2672</t>
+          <t>242 945 0171</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>david.moore@company.org</t>
+          <t>susan.miller@outlook.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10/9/1998</t>
+          <t>1994-05-14</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>5343 Oak St</t>
+          <t>3338 Cedar St</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>17576</t>
+          <t>77060</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>William Hernandez</t>
+          <t>Elizabeth Williams</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>761.337.5679</t>
+          <t>492 504 1925</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>william.hernandez@yahoo.com</t>
+          <t>elizabeth.williams@gmail.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4-10-1985</t>
+          <t>1973-09-26</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1450 Main St</t>
+          <t>2772 Elm St</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>32548</t>
+          <t>68018</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Elizabeth Jones</t>
+          <t>Patricia Anderson</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>+13166260696</t>
+          <t>(332) 131-8321</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>elizabeth.jones@mail.co</t>
+          <t>patricia.anderson@company.org</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>02.01.1993</t>
+          <t>1998-02-18</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>7357 Elm St</t>
+          <t>4643 Main St</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>33156</t>
+          <t>96237</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karen Rodriguez</t>
+          <t>Thomas Gonzalez</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>(401) 934-0443</t>
+          <t>940-926-1386</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>karen.rodriguez@mail.co</t>
+          <t>thomas.gonzalez@company.org</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>03.08.2000</t>
+          <t>2004-01-24</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3207 Main St</t>
+          <t>5083 Cedar St</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>30866</t>
+          <t>16089</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Joseph Martin</t>
+          <t>Thomas Williams</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>+18411057632</t>
+          <t>658-111-5237</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>joseph.martin@company.org</t>
+          <t>thomas.williams@yahoo.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09/04/1963</t>
+          <t>1986-11-05</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>6331 Oak St</t>
+          <t>9878 Oak St</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1679,128 +1679,128 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>94873</t>
+          <t>37407</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jessica Thomas</t>
+          <t>Karen Davis</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>(314) 319-7207</t>
+          <t>250.285.2216</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>jessica.thomas@outlook.com</t>
+          <t>karen.davis@company.org</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>11.09.1984</t>
+          <t>1975-11-12</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>3410 Pine St</t>
+          <t>535 Pine St</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>59407</t>
+          <t>43982</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Linda Gonzalez</t>
+          <t>Richard Rodriguez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>433 611 1398</t>
+          <t>741 323 7159</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>linda.gonzalez@gmail.com</t>
+          <t>richard.rodriguez@company.org</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1976-08-26</t>
+          <t>1994-11-18</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>5397 Cedar St</t>
+          <t>8794 Elm St</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>38785</t>
+          <t>61713</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Susan Moore</t>
+          <t>Susan Miller</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>248 294 3454</t>
+          <t>248 100 6624</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>susan.moore@mail.co</t>
+          <t>susan.miller@company.org</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>17.10.1986</t>
+          <t>1969-09-10</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>9237 Cedar St</t>
+          <t>1975 Elm St</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1810,34 +1810,34 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>17860</t>
+          <t>43743</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>William Moore</t>
+          <t>John Hernandez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>502.187.7420</t>
+          <t>555 358 3398</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>william.moore@company.org</t>
+          <t>john.hernandez@mail.co</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>03/07/1998</t>
+          <t>1992-05-05</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>6176 Elm St</t>
+          <t>3694 Cedar St</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1847,86 +1847,86 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>90694</t>
+          <t>21799</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Barbara Anderson</t>
+          <t>Joseph Johnson</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>968-825-9925</t>
+          <t>(398) 446-4299</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>barbara.anderson@company.org</t>
+          <t>joseph.johnson@gmail.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>25-11-1990</t>
+          <t>1961-12-21</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>8004 Main St</t>
+          <t>6345 Elm St</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>11578</t>
+          <t>79554</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Elizabeth Brown</t>
+          <t>John Gonzalez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>649.500.0014</t>
+          <t>(797) 274-2229</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>elizabeth.brown@mail.co</t>
+          <t>john.gonzalez@gmail.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>01/12/1965</t>
+          <t>2001-08-14</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>5591 Main St</t>
+          <t>3924 Main St</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1936,118 +1936,118 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>15941</t>
+          <t>93901</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Robert Gonzalez</t>
+          <t>Karen Williams</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>582.945.7550</t>
+          <t>462.793.0875</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>robert.gonzalez@company.org</t>
+          <t>karen.williams@outlook.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>11/16/1987</t>
+          <t>1993-10-05</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2774 Cedar St</t>
+          <t>8818 Cedar St</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>13057</t>
+          <t>91820</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>David Rodriguez</t>
+          <t>Susan Hernandez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>687-241-5807</t>
+          <t>805 329 7232</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>david.rodriguez@mail.co</t>
+          <t>susan.hernandez@yahoo.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10/27/1993</t>
+          <t>1991-08-25</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>209 Cedar St</t>
+          <t>2583 Main St</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>26969</t>
+          <t>81299</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Patricia Lopez</t>
+          <t>William Wilson</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>340-498-8557</t>
+          <t>(755) 609-7009</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>patricia.lopez@outlook.com</t>
+          <t>william.wilson@company.org</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>19-11-1992</t>
+          <t>1993-01-24</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>8736 Pine St</t>
+          <t>9219 Main St</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2057,44 +2057,44 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>57783</t>
+          <t>71953</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Thomas Thomas</t>
+          <t>Karen Johnson</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>635-184-5356</t>
+          <t>888.541.6080</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>thomas.thomas@mail.co</t>
+          <t>karen.johnson@company.org</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>07/20/1976</t>
+          <t>1983-06-26</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>8701 Oak St</t>
+          <t>5088 Pine St</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2104,34 +2104,34 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>51494</t>
+          <t>60922</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Barbara Rodriguez</t>
+          <t>Richard Martinez</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>+12488017774</t>
+          <t>738 544 1166</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>barbara.rodriguez@gmail.com</t>
+          <t>richard.martinez@outlook.com</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1970-05-04</t>
+          <t>1983-10-08</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>7903 Main St</t>
+          <t>7138 Elm St</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2141,123 +2141,123 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>36860</t>
+          <t>26634</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Susan Rodriguez</t>
+          <t>Jennifer Davis</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>297 377 3393</t>
+          <t>772 304 6867</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>susan.rodriguez@mail.co</t>
+          <t>jennifer.davis@mail.co</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>9-10-1971</t>
+          <t>1976-08-10</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2448 Elm St</t>
+          <t>6688 Pine St</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>70089</t>
+          <t>95407</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Barbara Taylor</t>
+          <t>Joseph Jones</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>788.194.6596</t>
+          <t>588.512.9050</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>barbara.taylor@mail.co</t>
+          <t>joseph.jones@yahoo.com</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10/28/1996</t>
+          <t>1968-10-13</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2046 Elm St</t>
+          <t>968 Cedar St</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>40707</t>
+          <t>79207</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Richard Davis</t>
+          <t>Jessica Moore</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>+19427622289</t>
+          <t>431 975 0471</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>richard.davis@mail.co</t>
+          <t>jessica.moore@yahoo.com</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>23-1-1997</t>
+          <t>1994-08-15</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>7764 Main St</t>
+          <t>6484 Oak St</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2267,212 +2267,212 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>25330</t>
+          <t>83028</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jennifer Martinez</t>
+          <t>Thomas Hernandez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>266.249.0365</t>
+          <t>(449) 629-9471</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>jennifer.martinez@yahoo.com</t>
+          <t>thomas.hernandez@outlook.com</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/04/1997</t>
+          <t>1990-09-19</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>5793 Oak St</t>
+          <t>5996 Main St</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>73876</t>
+          <t>36817</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Elizabeth Miller</t>
+          <t>Jennifer Martin</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>(453) 751-0865</t>
+          <t>504-571-8988</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>elizabeth.miller@outlook.com</t>
+          <t>jennifer.martin@mail.co</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1/22/2005</t>
+          <t>1961-12-27</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4240 Pine St</t>
+          <t>8227 Elm St</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>66703</t>
+          <t>13729</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Karen Thomas</t>
+          <t>Michael Thomas</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>(266) 504-3485</t>
+          <t>(371) 709-8665</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>karen.thomas@company.org</t>
+          <t>michael.thomas@mail.co</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>02/23/1972</t>
+          <t>1995-08-08</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2902 Elm St</t>
+          <t>9772 Main St</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>25494</t>
+          <t>45434</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mary Thomas</t>
+          <t>John Jones</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>750.462.2671</t>
+          <t>(526) 769-4426</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>mary.thomas@mail.co</t>
+          <t>john.jones@company.org</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>28-10-1980</t>
+          <t>1964-04-04</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>9156 Elm St</t>
+          <t>2251 Cedar St</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>73534</t>
+          <t>97565</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>Thomas Thomas</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>565-815-0254</t>
+          <t>(904) 947-6846</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sarah.johnson@gmail.com</t>
+          <t>thomas.thomas@yahoo.com</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>11/09/1965</t>
+          <t>2002-06-10</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>8138 Pine St</t>
+          <t>3229 Elm St</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2482,39 +2482,39 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>15043</t>
+          <t>54356</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Susan Garcia</t>
+          <t>Jessica Miller</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>256-381-2343</t>
+          <t>410-117-8776</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>susan.garcia@company.org</t>
+          <t>jessica.miller@gmail.com</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1997-08-02</t>
+          <t>1975-06-21</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>3832 Main St</t>
+          <t>2446 Main St</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2524,76 +2524,76 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>69477</t>
+          <t>49343</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>James Lopez</t>
+          <t>Barbara Martin</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>+13253615374</t>
+          <t>672 119 9681</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>james.lopez@gmail.com</t>
+          <t>barbara.martin@outlook.com</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>11/1/1961</t>
+          <t>1979-11-28</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>8203 Elm St</t>
+          <t>6788 Oak St</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>63322</t>
+          <t>60730</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Christopher Anderson</t>
+          <t>Richard Gonzalez</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>393 513 4169</t>
+          <t>859 469 1933</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>christopher.anderson@gmail.com</t>
+          <t>richard.gonzalez@yahoo.com</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2/15/2001</t>
+          <t>1974-03-07</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>205 Oak St</t>
+          <t>8144 Elm St</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2603,86 +2603,86 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>83602</t>
+          <t>13966</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>John Martin</t>
+          <t>Karen Smith</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>(619) 314-1187</t>
+          <t>(621) 242-5680</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>john.martin@mail.co</t>
+          <t>karen.smith@yahoo.com</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>5-11-1971</t>
+          <t>2004-03-22</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1903 Elm St</t>
+          <t>1416 Pine St</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>33550</t>
+          <t>96615</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>William Thomas</t>
+          <t>Susan Martinez</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>(631) 197-7950</t>
+          <t>880-511-9366</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>william.thomas@yahoo.com</t>
+          <t>susan.martinez@mail.co</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>12/2/1978</t>
+          <t>1999-07-13</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>562 Main St</t>
+          <t>8734 Cedar St</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2692,291 +2692,291 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>49010</t>
+          <t>49124</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>James Moore</t>
+          <t>John Moore</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>951-999-5788</t>
+          <t>909-346-3632</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>james.moore@mail.co</t>
+          <t>john.moore@yahoo.com</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10/11/1995</t>
+          <t>1985-11-07</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>9050 Cedar St</t>
+          <t>1977 Pine St</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>80273</t>
+          <t>68950</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Sarah Thomas</t>
+          <t>Karen Garcia</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>786 878 5440</t>
+          <t>668-210-2571</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sarah.thomas@mail.co</t>
+          <t>karen.garcia@yahoo.com</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1982-04-14</t>
+          <t>1995-10-25</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>5509 Oak St</t>
+          <t>3481 Pine St</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>87225</t>
+          <t>85332</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>David Garcia</t>
+          <t>Sarah Jackson</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>+14184765024</t>
+          <t>(202) 426-5967</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>david.garcia@outlook.com</t>
+          <t>sarah.jackson@mail.co</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>26-2-1963</t>
+          <t>1993-08-22</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>6169 Cedar St</t>
+          <t>1384 Pine St</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>96821</t>
+          <t>42334</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Linda Martin</t>
+          <t>Christopher Hernandez</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>665-888-8633</t>
+          <t>(781) 717-5535</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>linda.martin@outlook.com</t>
+          <t>christopher.hernandez@yahoo.com</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>9/5/1963</t>
+          <t>1992-01-17</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>9987 Cedar St</t>
+          <t>2593 Main St</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>13801</t>
+          <t>18307</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Jessica Williams</t>
+          <t>Sarah Moore</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>308 352 4293</t>
+          <t>466.828.6316</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>jessica.williams@gmail.com</t>
+          <t>sarah.moore@yahoo.com</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10/18/1992</t>
+          <t>1981-11-11</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>3413 Main St</t>
+          <t>8947 Pine St</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>77126</t>
+          <t>94936</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>William Wilson</t>
+          <t>Linda Smith</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>+17805351627</t>
+          <t>(201) 894-7056</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>william.wilson@yahoo.com</t>
+          <t>linda.smith@outlook.com</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>04/16/1961</t>
+          <t>1983-11-20</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>760 Oak St</t>
+          <t>9227 Elm St</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>52619</t>
+          <t>35515</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>William Anderson</t>
+          <t>Barbara Smith</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>(613) 222-9924</t>
+          <t>(594) 492-6933</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>william.anderson@outlook.com</t>
+          <t>barbara.smith@company.org</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>06.02.1981</t>
+          <t>1961-03-20</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>9657 Pine St</t>
+          <t>7056 Oak St</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2986,34 +2986,34 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>23605</t>
+          <t>16030</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Linda Brown</t>
+          <t>John Taylor</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>878.610.7197</t>
+          <t>(594) 912-6275</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>linda.brown@mail.co</t>
+          <t>john.taylor@gmail.com</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>20.10.1985</t>
+          <t>2003-08-04</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>4870 Main St</t>
+          <t>6808 Oak St</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3023,39 +3023,39 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>22536</t>
+          <t>30138</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>James Jones</t>
+          <t>Christopher Lopez</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>531.484.2195</t>
+          <t>(449) 859-6736</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>james.jones@gmail.com</t>
+          <t>christopher.lopez@gmail.com</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>1979-12-25</t>
+          <t>1979-01-07</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>3091 Pine St</t>
+          <t>5980 Pine St</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3065,165 +3065,165 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>11148</t>
+          <t>14835</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>William Miller</t>
+          <t>Robert Anderson</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>+14931474540</t>
+          <t>(790) 416-9498</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>william.miller@gmail.com</t>
+          <t>robert.anderson@mail.co</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>1983-04-22</t>
+          <t>2000-03-08</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>7527 Elm St</t>
+          <t>7514 Pine St</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>23928</t>
+          <t>44216</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Christopher Moore</t>
+          <t>Sarah Anderson</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>399 734 5945</t>
+          <t>298 500 1295</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>christopher.moore@gmail.com</t>
+          <t>sarah.anderson@gmail.com</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>01.06.1979</t>
+          <t>1980-04-28</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>7866 Pine St</t>
+          <t>5776 Elm St</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>54966</t>
+          <t>74835</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Robert Martin</t>
+          <t>Jennifer Thomas</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>397 604 7345</t>
+          <t>303 273 1948</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>robert.martin@outlook.com</t>
+          <t>jennifer.thomas@yahoo.com</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>1/1/1977</t>
+          <t>2004-11-17</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>9244 Main St</t>
+          <t>6650 Elm St</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>56152</t>
+          <t>72426</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Robert Davis</t>
+          <t>Susan Davis</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>488.262.8147</t>
+          <t>(849) 235-6254</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>robert.davis@company.org</t>
+          <t>susan.davis@yahoo.com</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>18.05.1984</t>
+          <t>1981-04-26</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>3142 Cedar St</t>
+          <t>5995 Elm St</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3238,34 +3238,34 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>23158</t>
+          <t>21377</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>David Martin</t>
+          <t>Karen Gonzalez</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>856.899.3986</t>
+          <t>319-354-8661</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>david.martin@company.org</t>
+          <t>karen.gonzalez@mail.co</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>1987-10-18</t>
+          <t>1987-12-21</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>4327 Oak St</t>
+          <t>2405 Cedar St</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3275,170 +3275,170 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>83289</t>
+          <t>42072</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Jennifer Hernandez</t>
+          <t>Thomas Smith</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>+16554271106</t>
+          <t>(849) 588-1480</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>jennifer.hernandez@company.org</t>
+          <t>thomas.smith@outlook.com</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>17-5-1985</t>
+          <t>1994-02-05</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1655 Cedar St</t>
+          <t>6388 Pine St</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>37818</t>
+          <t>62199</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Joseph Moore</t>
+          <t>William Rodriguez</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>364.906.7048</t>
+          <t>903.609.5813</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>joseph.moore@outlook.com</t>
+          <t>william.rodriguez@outlook.com</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>1970-03-07</t>
+          <t>1995-01-13</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>7062 Oak St</t>
+          <t>6545 Cedar St</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>77479</t>
+          <t>39846</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>James Martinez</t>
+          <t>Michael Williams</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>(923) 402-6166</t>
+          <t>(513) 906-5029</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>james.martinez@mail.co</t>
+          <t>michael.williams@mail.co</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>8/17/1995</t>
+          <t>1997-08-03</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>9735 Oak St</t>
+          <t>9804 Main St</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>53190</t>
+          <t>10136</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Elizabeth Anderson</t>
+          <t>Sarah Brown</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>749 714 2215</t>
+          <t>646 123 1727</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>elizabeth.anderson@mail.co</t>
+          <t>sarah.brown@company.org</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2004-11-01</t>
+          <t>2005-08-28</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>8017 Elm St</t>
+          <t>4656 Main St</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3448,34 +3448,34 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>89372</t>
+          <t>47040</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Thomas Taylor</t>
+          <t>David Davis</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>+14205170762</t>
+          <t>(429) 522-1173</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>thomas.taylor@mail.co</t>
+          <t>david.davis@gmail.com</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>1981-07-28</t>
+          <t>1969-05-12</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>909 Cedar St</t>
+          <t>6387 Elm St</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3485,44 +3485,44 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>35720</t>
+          <t>32618</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Linda Williams</t>
+          <t>Linda Wilson</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>212-595-2427</t>
+          <t>(340) 319-7317</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>linda.williams@company.org</t>
+          <t>linda.wilson@gmail.com</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>19-8-1974</t>
+          <t>1996-12-12</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>3234 Cedar St</t>
+          <t>2886 Elm St</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3532,207 +3532,207 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>59464</t>
+          <t>71457</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Michael Anderson</t>
+          <t>Jessica Taylor</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>274-361-8010</t>
+          <t>471 485 9552</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>michael.anderson@gmail.com</t>
+          <t>jessica.taylor@outlook.com</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>6/9/2001</t>
+          <t>1985-09-19</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>7527 Elm St</t>
+          <t>2820 Elm St</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>83555</t>
+          <t>82631</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Patricia Lopez</t>
+          <t>Christopher Johnson</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>+16604477231</t>
+          <t>(798) 192-5562</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>patricia.lopez@yahoo.com</t>
+          <t>christopher.johnson@gmail.com</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>14.03.1979</t>
+          <t>1978-03-22</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>7795 Main St</t>
+          <t>7249 Pine St</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>70059</t>
+          <t>25103</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Mary Martin</t>
+          <t>Patricia Gonzalez</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>744-412-7830</t>
+          <t>540-777-1221</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>mary.martin@outlook.com</t>
+          <t>patricia.gonzalez@outlook.com</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>6/16/1992</t>
+          <t>1974-03-25</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>4149 Elm St</t>
+          <t>1979 Cedar St</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>90198</t>
+          <t>45854</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Thomas Wilson</t>
+          <t>John Jones</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>(975) 350-5312</t>
+          <t>(467) 821-1335</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>thomas.wilson@company.org</t>
+          <t>john.jones@outlook.com</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>23-8-1995</t>
+          <t>1963-03-09</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>4910 Cedar St</t>
+          <t>8884 Pine St</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>99917</t>
+          <t>65230</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Linda Moore</t>
+          <t>William Davis</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>893-535-9440</t>
+          <t>968.760.3113</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>linda.moore@outlook.com</t>
+          <t>william.davis@company.org</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>18.12.1978</t>
+          <t>1995-12-18</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2300 Main St</t>
+          <t>2760 Cedar St</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3742,118 +3742,118 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>69582</t>
+          <t>99675</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Susan Taylor</t>
+          <t>Susan Martin</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>749.681.2582</t>
+          <t>815.490.2602</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>susan.taylor@yahoo.com</t>
+          <t>susan.martin@gmail.com</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>25.10.1960</t>
+          <t>1987-08-05</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>8176 Elm St</t>
+          <t>5847 Elm St</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>62712</t>
+          <t>28289</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Jessica Smith</t>
+          <t>David Martin</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>292.735.2890</t>
+          <t>944.507.4519</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>jessica.smith@gmail.com</t>
+          <t>david.martin@yahoo.com</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>1999-02-28</t>
+          <t>1986-06-15</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>6858 Elm St</t>
+          <t>6743 Pine St</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>79865</t>
+          <t>92470</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Richard Garcia</t>
+          <t>Thomas Anderson</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>+15567874859</t>
+          <t>793.798.7549</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>richard.garcia@yahoo.com</t>
+          <t>thomas.anderson@company.org</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>14.02.1967</t>
+          <t>1976-10-26</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>8118 Main St</t>
+          <t>4111 Elm St</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3863,123 +3863,123 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>49924</t>
+          <t>92256</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>James Thomas</t>
+          <t>Karen Johnson</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>980-202-1410</t>
+          <t>639-352-8970</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>james.thomas@mail.co</t>
+          <t>karen.johnson@outlook.com</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>9-8-2000</t>
+          <t>1966-08-09</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>3719 Oak St</t>
+          <t>2843 Pine St</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>96720</t>
+          <t>84178</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Karen Martin</t>
+          <t>Mary Lopez</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>(297) 489-5856</t>
+          <t>(217) 626-4398</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>karen.martin@company.org</t>
+          <t>mary.lopez@company.org</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>1987-10-09</t>
+          <t>1995-05-13</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2282 Pine St</t>
+          <t>3489 Oak St</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>49778</t>
+          <t>81774</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Richard Jackson</t>
+          <t>Robert Hernandez</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>(495) 789-1511</t>
+          <t>(818) 155-0188</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>richard.jackson@gmail.com</t>
+          <t>robert.hernandez@gmail.com</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2-7-1972</t>
+          <t>1978-03-05</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>4997 Elm St</t>
+          <t>8390 Main St</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3989,44 +3989,44 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>22536</t>
+          <t>67478</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Thomas Johnson</t>
+          <t>Mary Jackson</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>+19498792139</t>
+          <t>(383) 642-3582</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>thomas.johnson@company.org</t>
+          <t>mary.jackson@outlook.com</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>24-11-1982</t>
+          <t>1980-12-12</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>8557 Cedar St</t>
+          <t>5160 Oak St</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4036,123 +4036,123 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>32517</t>
+          <t>64413</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Patricia Johnson</t>
+          <t>Elizabeth Jones</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>705.982.7162</t>
+          <t>239 514 0612</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>patricia.johnson@company.org</t>
+          <t>elizabeth.jones@company.org</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>06/15/1986</t>
+          <t>1966-07-07</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>6365 Pine St</t>
+          <t>8137 Pine St</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>29009</t>
+          <t>95357</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Thomas Gonzalez</t>
+          <t>Christopher Garcia</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>+13763952213</t>
+          <t>291.949.2387</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>thomas.gonzalez@company.org</t>
+          <t>christopher.garcia@mail.co</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>8/12/1976</t>
+          <t>1994-08-05</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>7921 Main St</t>
+          <t>5809 Oak St</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>56196</t>
+          <t>44648</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Jessica Hernandez</t>
+          <t>Barbara Garcia</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>622.183.7907</t>
+          <t>(768) 759-7377</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>jessica.hernandez@outlook.com</t>
+          <t>barbara.garcia@yahoo.com</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>1962-01-28</t>
+          <t>1964-08-04</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>3639 Elm St</t>
+          <t>7206 Main St</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4162,76 +4162,76 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>42094</t>
+          <t>45795</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Thomas Gonzalez</t>
+          <t>Joseph Smith</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>266-428-9076</t>
+          <t>902.861.4442</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>thomas.gonzalez@yahoo.com</t>
+          <t>joseph.smith@mail.co</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>26-12-1971</t>
+          <t>1998-05-11</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>9911 Cedar St</t>
+          <t>8616 Oak St</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>41326</t>
+          <t>59929</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Thomas Wilson</t>
+          <t>Sarah Taylor</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>674-163-0788</t>
+          <t>884 150 8640</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>thomas.wilson@company.org</t>
+          <t>sarah.taylor@yahoo.com</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>06/25/2001</t>
+          <t>1990-04-17</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>6968 Pine St</t>
+          <t>2840 Cedar St</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4241,165 +4241,165 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>53337</t>
+          <t>41484</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Linda Williams</t>
+          <t>Richard Smith</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>+13967454878</t>
+          <t>388.749.2617</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>linda.williams@mail.co</t>
+          <t>richard.smith@mail.co</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>11/26/2001</t>
+          <t>2000-03-14</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>9718 Pine St</t>
+          <t>9322 Oak St</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>28475</t>
+          <t>78878</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>David Taylor</t>
+          <t>William Gonzalez</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>755.865.8569</t>
+          <t>(348) 190-6393</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>david.taylor@mail.co</t>
+          <t>william.gonzalez@gmail.com</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>11/03/1967</t>
+          <t>1978-01-16</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>1597 Oak St</t>
+          <t>7097 Elm St</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>93435</t>
+          <t>34632</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>James Jackson</t>
+          <t>James Rodriguez</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>484-105-4811</t>
+          <t>961 986 7175</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>james.jackson@outlook.com</t>
+          <t>james.rodriguez@mail.co</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>9-9-1979</t>
+          <t>1962-09-08</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>4374 Pine St</t>
+          <t>5037 Elm St</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>90848</t>
+          <t>70537</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Jessica Jones</t>
+          <t>Mary Miller</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>+15898542982</t>
+          <t>437.688.9349</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>jessica.jones@yahoo.com</t>
+          <t>mary.miller@yahoo.com</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>17-3-1990</t>
+          <t>1975-01-05</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>95 Oak St</t>
+          <t>4425 Main St</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4409,254 +4409,254 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>29734</t>
+          <t>93498</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Linda Martin</t>
+          <t>Patricia Smith</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>307 195 6534</t>
+          <t>(666) 743-8248</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>linda.martin@gmail.com</t>
+          <t>patricia.smith@yahoo.com</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>1/5/1967</t>
+          <t>1978-02-26</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>8672 Pine St</t>
+          <t>4192 Pine St</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>22806</t>
+          <t>62095</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Christopher Jackson</t>
+          <t>Patricia Lopez</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>218-450-8275</t>
+          <t>619 488 0549</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>christopher.jackson@gmail.com</t>
+          <t>patricia.lopez@yahoo.com</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>01/25/1996</t>
+          <t>1996-06-05</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>5615 Main St</t>
+          <t>4868 Main St</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>14763</t>
+          <t>51805</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Patricia Hernandez</t>
+          <t>Linda Martin</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>547-660-6314</t>
+          <t>222 509 8682</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>patricia.hernandez@company.org</t>
+          <t>linda.martin@yahoo.com</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>20.02.1999</t>
+          <t>1988-01-28</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>7268 Oak St</t>
+          <t>3054 Pine St</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>51235</t>
+          <t>88349</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Jennifer Davis</t>
+          <t>Elizabeth Williams</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>(350) 616-5174</t>
+          <t>(890) 751-4705</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>jennifer.davis@outlook.com</t>
+          <t>elizabeth.williams@outlook.com</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>06.11.1990</t>
+          <t>1973-08-23</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>1442 Cedar St</t>
+          <t>3775 Elm St</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>40291</t>
+          <t>93493</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Robert Garcia</t>
+          <t>Robert Jones</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>440.427.6204</t>
+          <t>851 336 8052</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>robert.garcia@mail.co</t>
+          <t>robert.jones@outlook.com</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>5-7-1976</t>
+          <t>2000-08-28</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>3282 Oak St</t>
+          <t>9211 Oak St</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>90928</t>
+          <t>75377</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Karen Williams</t>
+          <t>Karen Thomas</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>954.591.8296</t>
+          <t>750 786 6574</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>karen.williams@gmail.com</t>
+          <t>karen.thomas@gmail.com</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>27-1-1974</t>
+          <t>1976-12-20</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>1515 Cedar St</t>
+          <t>8362 Oak St</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>93604</t>
+          <t>69895</t>
         </is>
       </c>
     </row>

</xml_diff>